<commit_message>
Update to only show C2 scenario
</commit_message>
<xml_diff>
--- a/input_data/flow_scen/FallFlows20260909_Draft.xlsx
+++ b/input_data/flow_scen/FallFlows20260909_Draft.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/lelliott_usbr_gov/Documents/Documents/GitHub/BDO-Science/Fall_Flow_Redd_Dewatering/input_data/flow_scen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E7DFD7F7-14B9-49AC-881D-4D1AA1487E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{E7DFD7F7-14B9-49AC-881D-4D1AA1487E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DB0ECA0-42DC-4E7B-8171-0748776191AF}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="876" xr2:uid="{8B6B0201-DD1B-4D0A-8FA2-1793C828B1EC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="876" activeTab="1" xr2:uid="{8B6B0201-DD1B-4D0A-8FA2-1793C828B1EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Keswick Flow Alternatives" sheetId="3" r:id="rId1"/>
@@ -1831,40 +1831,40 @@
                   <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="41">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="42">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="43">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="44">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="45">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="46">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="47">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="48">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="49">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="50">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>10000000</c:v>
+                  <c:v>-100</c:v>
                 </c:pt>
                 <c:pt idx="52">
                   <c:v>10000000</c:v>
@@ -14188,7 +14188,7 @@
       <c r="O43" s="1"/>
       <c r="P43">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.3">
@@ -14226,7 +14226,7 @@
       <c r="O44" s="1"/>
       <c r="P44">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.3">
@@ -14264,7 +14264,7 @@
       <c r="O45" s="1"/>
       <c r="P45">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.3">
@@ -14302,7 +14302,7 @@
       <c r="O46" s="1"/>
       <c r="P46">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
@@ -14340,7 +14340,7 @@
       <c r="O47" s="1"/>
       <c r="P47">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.3">
@@ -14378,7 +14378,7 @@
       <c r="O48" s="1"/>
       <c r="P48">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
@@ -14416,7 +14416,7 @@
       <c r="O49" s="1"/>
       <c r="P49">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.3">
@@ -14454,7 +14454,7 @@
       <c r="O50" s="1"/>
       <c r="P50">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.3">
@@ -14492,7 +14492,7 @@
       <c r="O51" s="1"/>
       <c r="P51">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.3">
@@ -14530,7 +14530,7 @@
       <c r="O52" s="1"/>
       <c r="P52">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.3">
@@ -14568,7 +14568,7 @@
       <c r="O53" s="1"/>
       <c r="P53">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.3">
@@ -14606,7 +14606,7 @@
       <c r="O54" s="1"/>
       <c r="P54">
         <f t="shared" ca="1" si="0"/>
-        <v>10000000</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.3">
@@ -21697,7 +21697,7 @@
         <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>